<commit_message>
Add image viewer pages
</commit_message>
<xml_diff>
--- a/Digital_Twin_Report.xlsx
+++ b/Digital_Twin_Report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjakhema\Downloads\Level3DViews_CLIENT_PACKAGE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://my.jci.com/sites/BIMProjectData/Shared Documents/01. BIM Project Data/01. Digital Twin Projects/Digital Twin Project/01_Mayui Trial Project/Level3DViews_CLIENT_PACKAGE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF0FAEB-23FF-4D3E-8257-7AEF6B2B1949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_123110AED330D3583920D5F0505ED87656CD17CF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{472B4EFC-C904-4DAE-9109-F95C5608F585}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="34605" yWindow="0" windowWidth="22110" windowHeight="14700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -108,7 +108,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,38 +116,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -155,34 +133,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -483,447 +441,709 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="3" t="str">
+      <c r="D2" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_2-MJ 2_25/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E2" s="3" t="str">
+      <c r="E2" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_2-MJ 2_25","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F2" s="3" t="str">
+      <c r="F2" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_2-MJ 2_25/DT_MJ_2-MJ 2_25.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G2" s="3" t="str">
+      <c r="G2" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_2-MJ 2_25/DT_MJ_2-MJ 2_25_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H2" s="3" t="str">
+      <c r="H2" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_2-MJ 2_25/DT_MJ_2-MJ 2_25_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I2" s="3" t="str">
+      <c r="I2" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_2-MJ 2_25/DT_MJ_2-MJ 2_25_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="str">
+      <c r="D3" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_3-MJ 2_25/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E3" s="3" t="str">
+      <c r="E3" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_3-MJ 2_25","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F3" s="3" t="str">
+      <c r="F3" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_3-MJ 2_25/DT_MJ_3-MJ 2_25.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G3" s="3" t="str">
+      <c r="G3" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_3-MJ 2_25/DT_MJ_3-MJ 2_25_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H3" s="3" t="str">
+      <c r="H3" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_3-MJ 2_25/DT_MJ_3-MJ 2_25_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I3" s="3" t="str">
+      <c r="I3" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_3-MJ 2_25/DT_MJ_3-MJ 2_25_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="3" t="str">
+      <c r="D4" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_4-MJ 2_25/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E4" s="3" t="str">
+      <c r="E4" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_4-MJ 2_25","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F4" s="3" t="str">
+      <c r="F4" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_4-MJ 2_25/DT_MJ_4-MJ 2_25.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G4" s="3" t="str">
+      <c r="G4" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_4-MJ 2_25/DT_MJ_4-MJ 2_25_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H4" s="3" t="str">
+      <c r="H4" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_4-MJ 2_25/DT_MJ_4-MJ 2_25_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I4" s="3" t="str">
+      <c r="I4" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_4-MJ 2_25/DT_MJ_4-MJ 2_25_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3" t="str">
+      <c r="D5" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_5-MJ 2_25/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E5" s="3" t="str">
+      <c r="E5" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_5-MJ 2_25","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F5" s="3" t="str">
+      <c r="F5" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_5-MJ 2_25/DT_MJ_5-MJ 2_25.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G5" s="3" t="str">
+      <c r="G5" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_5-MJ 2_25/DT_MJ_5-MJ 2_25_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H5" s="3" t="str">
+      <c r="H5" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_5-MJ 2_25/DT_MJ_5-MJ 2_25_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I5" s="3" t="str">
+      <c r="I5" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_5-MJ 2_25/DT_MJ_5-MJ 2_25_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="3" t="str">
+      <c r="D6" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_6-MJ 2_25/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E6" s="3" t="str">
+      <c r="E6" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_6-MJ 2_25","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F6" s="3" t="str">
+      <c r="F6" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_6-MJ 2_25/DT_MJ_6-MJ 2_25.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G6" s="3" t="str">
+      <c r="G6" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_6-MJ 2_25/DT_MJ_6-MJ 2_25_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H6" s="3" t="str">
+      <c r="H6" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_6-MJ 2_25/DT_MJ_6-MJ 2_25_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I6" s="3" t="str">
+      <c r="I6" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_6-MJ 2_25/DT_MJ_6-MJ 2_25_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="3" t="str">
+      <c r="D7" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_7-MJ 2_25/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E7" s="3" t="str">
+      <c r="E7" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_7-MJ 2_25","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F7" s="3" t="str">
+      <c r="F7" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_7-MJ 2_25/DT_MJ_7-MJ 2_25.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G7" s="3" t="str">
+      <c r="G7" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_7-MJ 2_25/DT_MJ_7-MJ 2_25_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H7" s="3" t="str">
+      <c r="H7" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_7-MJ 2_25/DT_MJ_7-MJ 2_25_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I7" s="3" t="str">
+      <c r="I7" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_7-MJ 2_25/DT_MJ_7-MJ 2_25_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="3" t="str">
+      <c r="D8" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_8-MJ 2_25/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E8" s="3" t="str">
+      <c r="E8" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_8-MJ 2_25","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F8" s="3" t="str">
+      <c r="F8" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_8-MJ 2_25/DT_MJ_8-MJ 2_25.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G8" s="3" t="str">
+      <c r="G8" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_8-MJ 2_25/DT_MJ_8-MJ 2_25_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H8" s="3" t="str">
+      <c r="H8" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_8-MJ 2_25/DT_MJ_8-MJ 2_25_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I8" s="3" t="str">
+      <c r="I8" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 2_25/DT_MJ_8-MJ 2_25/DT_MJ_8-MJ 2_25_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="3" t="str">
+      <c r="D9" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_31-MJ 7_21/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E9" s="3" t="str">
+      <c r="E9" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_31-MJ 7_21","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F9" s="3" t="str">
+      <c r="F9" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_31-MJ 7_21/DT_MJ_31-MJ 7_21.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G9" s="3" t="str">
+      <c r="G9" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_31-MJ 7_21/DT_MJ_31-MJ 7_21_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H9" s="3" t="str">
+      <c r="H9" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_31-MJ 7_21/DT_MJ_31-MJ 7_21_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I9" s="3" t="str">
+      <c r="I9" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_31-MJ 7_21/DT_MJ_31-MJ 7_21_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="3" t="str">
+      <c r="D10" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_32-MJ 7_21/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E10" s="3" t="str">
+      <c r="E10" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_32-MJ 7_21","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F10" s="3" t="str">
+      <c r="F10" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_32-MJ 7_21/DT_MJ_32-MJ 7_21.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G10" s="3" t="str">
+      <c r="G10" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_32-MJ 7_21/DT_MJ_32-MJ 7_21_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H10" s="3" t="str">
+      <c r="H10" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_32-MJ 7_21/DT_MJ_32-MJ 7_21_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I10" s="3" t="str">
+      <c r="I10" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_32-MJ 7_21/DT_MJ_32-MJ 7_21_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="3" t="str">
+      <c r="D11" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_33-MJ 7_21/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E11" s="3" t="str">
+      <c r="E11" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_33-MJ 7_21","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F11" s="3" t="str">
+      <c r="F11" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_33-MJ 7_21/DT_MJ_33-MJ 7_21.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G11" s="3" t="str">
+      <c r="G11" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_33-MJ 7_21/DT_MJ_33-MJ 7_21_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H11" s="3" t="str">
+      <c r="H11" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_33-MJ 7_21/DT_MJ_33-MJ 7_21_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I11" s="3" t="str">
+      <c r="I11" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_33-MJ 7_21/DT_MJ_33-MJ 7_21_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="3" t="str">
+      <c r="D12" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_34-MJ 7_21/viewer.html","Open Viewer")</f>
         <v>Open Viewer</v>
       </c>
-      <c r="E12" s="3" t="str">
+      <c r="E12" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_34-MJ 7_21","Open Images")</f>
         <v>Open Images</v>
       </c>
-      <c r="F12" s="3" t="str">
+      <c r="F12" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_34-MJ 7_21/DT_MJ_34-MJ 7_21.mp4","Clean Video")</f>
         <v>Clean Video</v>
       </c>
-      <c r="G12" s="3" t="str">
+      <c r="G12" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_34-MJ 7_21/DT_MJ_34-MJ 7_21_M.mp4","Meta Video")</f>
         <v>Meta Video</v>
       </c>
-      <c r="H12" s="3" t="str">
+      <c r="H12" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_34-MJ 7_21/DT_MJ_34-MJ 7_21_C.mp4","Comp Video")</f>
         <v>Comp Video</v>
       </c>
-      <c r="I12" s="3" t="str">
+      <c r="I12" t="str">
         <f>HYPERLINK("./3D_Level 1_to_Level 2/MJ 7_21/DT_MJ_34-MJ 7_21/DT_MJ_34-MJ 7_21_CM.mp4","Meta Comp")</f>
         <v>Meta Comp</v>
       </c>
-      <c r="J12" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003AC403995C123248B06F82225AEB3A59" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="69656b2c18d8e55c2b14d39a6d5aa9d3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="299b3cfa-fb26-4c5d-960e-988bf4540ad2" xmlns:ns3="db6d8cc1-4f24-4dff-ac2a-ca3fdcf18f71" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="716ce87849d126ea9baa065c19036576" ns2:_="" ns3:_="">
+    <xsd:import namespace="299b3cfa-fb26-4c5d-960e-988bf4540ad2"/>
+    <xsd:import namespace="db6d8cc1-4f24-4dff-ac2a-ca3fdcf18f71"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:Remarks" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="299b3cfa-fb26-4c5d-960e-988bf4540ad2" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="f2a00314-ae30-474d-911b-f8e025e1af2d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Remarks" ma:index="23" nillable="true" ma:displayName="Remarks" ma:format="Dropdown" ma:internalName="Remarks">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="24" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="db6d8cc1-4f24-4dff-ac2a-ca3fdcf18f71" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{8b69f1b9-cf2d-4f61-ad72-e4236a7d093e}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="db6d8cc1-4f24-4dff-ac2a-ca3fdcf18f71">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Remarks xmlns="299b3cfa-fb26-4c5d-960e-988bf4540ad2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="299b3cfa-fb26-4c5d-960e-988bf4540ad2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="db6d8cc1-4f24-4dff-ac2a-ca3fdcf18f71" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0895A4C-6203-479A-9054-7E8DBBA1C1A7}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E9A70BB7-CABD-455F-9E49-65BA8D6B6F1A}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7464BA13-965C-4789-9908-F409CAD7F1C3}"/>
 </file>
</xml_diff>